<commit_message>
feat(item-search): BUILDER wave — 3 specs green x2, module run-all 39/39 (PRS 19 / PCD 10 / PGR 10); shared grid base + 3 page objects + 3 selector sets + data constants; fixes: keystroke-debounce commit window, popover attribute anchor, tooltip stage-clearing, filtered-list Enter-commit, span-level truncation instrument (TC-006 correction cycle swept MD/plan/inventory), history-tab hydration gate, product-type set order-agnostic; workbook rebuilt
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/encore/testcases/item-search/item-search-product-code.xlsx
+++ b/clients/encore/testcases/item-search/item-search-product-code.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="117">
   <si>
     <t>TC ID</t>
   </si>
@@ -76,21 +76,24 @@
     <t>Medium</t>
   </si>
   <si>
-    <t>Pending Automation</t>
+    <t>Automated</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>A default search has been executed on the Products page for office 1101</t>
+  </si>
+  <si>
+    <t>1. Click any result row</t>
+  </si>
+  <si>
+    <t>The row highlights as selected</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>A default search has been executed on the Products page for office 1101</t>
-  </si>
-  <si>
-    <t>1. Click any result row</t>
-  </si>
-  <si>
-    <t>The row highlights as selected</t>
-  </si>
-  <si>
     <t>2. Read the toolbar above the grid</t>
   </si>
   <si>
@@ -352,16 +355,16 @@
     <t>Item Search — Product Code</t>
   </si>
   <si>
-    <t>Automated: 0 / Pending: 10</t>
-  </si>
-  <si>
-    <t>Not run in this delivery</t>
+    <t>Automated: 10 / Pending: 0</t>
+  </si>
+  <si>
+    <t>Pass:10 Fail:0 Skipped:0 Blocked:0</t>
   </si>
   <si>
     <t>Last Updated: 2026-08-31</t>
   </si>
   <si>
-    <t>f28c807cfb6eeb8b94ac190190f1358c8dc4f8c37d5142ffe46b461a0507db07</t>
+    <t>d96ccb59875274442c18342f06a9aa9c3097f6ed8a4e1cb1fd5e32267acbe42c</t>
   </si>
 </sst>
 </file>
@@ -759,7 +762,7 @@
     <col min="5" max="5" width="80" customWidth="1"/>
     <col min="6" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="28" customWidth="1"/>
-    <col min="9" max="9" width="26" customWidth="1"/>
+    <col min="9" max="9" width="36" customWidth="1"/>
     <col min="10" max="10" width="73" customWidth="1"/>
     <col min="11" max="11" width="69" customWidth="1"/>
     <col min="12" max="12" width="80" customWidth="1"/>
@@ -845,56 +848,56 @@
         <v>24</v>
       </c>
       <c r="M2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F3" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G3" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H3" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I3" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J3" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M3" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
         <v>15</v>
@@ -918,188 +921,188 @@
         <v>21</v>
       </c>
       <c r="J4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M4" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="L5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="L7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="L8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="M8" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
         <v>15</v>
@@ -1123,106 +1126,106 @@
         <v>21</v>
       </c>
       <c r="J9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M9" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="L11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="M11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C12" t="s">
         <v>15</v>
@@ -1246,147 +1249,147 @@
         <v>21</v>
       </c>
       <c r="J12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="L12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M12" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C13" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D13" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E13" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F13" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G13" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H13" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I13" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J13" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M13" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D14" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E14" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F14" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G14" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H14" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I14" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J14" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="M14" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="L15" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="M15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B16" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C16" t="s">
         <v>15</v>
@@ -1410,147 +1413,147 @@
         <v>21</v>
       </c>
       <c r="J16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="L16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="M16" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C17" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D17" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E17" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F17" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G17" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H17" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I17" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J17" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K17" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M17" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C18" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D18" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E18" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F18" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G18" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H18" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I18" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J18" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="L18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M18" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C19" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D19" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E19" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F19" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G19" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H19" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I19" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J19" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="L19" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="M19" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B20" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C20" t="s">
         <v>15</v>
@@ -1574,147 +1577,147 @@
         <v>21</v>
       </c>
       <c r="J20" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K20" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="L20" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="M20" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C21" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D21" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E21" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F21" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G21" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H21" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I21" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J21" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K21" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="L21" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="M21" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C22" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D22" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E22" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F22" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G22" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H22" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I22" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J22" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="M22" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C23" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D23" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E23" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F23" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G23" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H23" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I23" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J23" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K23" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="L23" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="M23" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B24" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C24" t="s">
         <v>15</v>
@@ -1738,147 +1741,147 @@
         <v>21</v>
       </c>
       <c r="J24" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K24" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="L24" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="M24" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B25" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C25" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D25" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E25" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F25" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G25" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H25" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I25" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J25" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K25" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="L25" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M25" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C26" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D26" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E26" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F26" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G26" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H26" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I26" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J26" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K26" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="L26" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="M26" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C27" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D27" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E27" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F27" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G27" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H27" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I27" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J27" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K27" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="L27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="M27" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B28" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C28" t="s">
         <v>15</v>
@@ -1902,106 +1905,106 @@
         <v>21</v>
       </c>
       <c r="J28" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K28" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="L28" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="M28" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B29" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C29" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D29" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E29" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F29" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G29" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H29" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I29" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J29" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K29" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L29" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M29" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B30" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C30" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D30" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E30" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F30" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G30" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H30" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I30" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J30" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L30" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="M30" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B31" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C31" t="s">
         <v>15</v>
@@ -2025,147 +2028,147 @@
         <v>21</v>
       </c>
       <c r="J31" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K31" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L31" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="M31" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B32" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C32" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D32" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E32" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F32" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G32" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H32" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I32" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J32" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K32" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L32" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M32" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B33" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C33" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D33" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E33" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F33" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G33" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H33" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I33" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J33" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K33" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L33" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="M33" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B34" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C34" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D34" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E34" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F34" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G34" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H34" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I34" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J34" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K34" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="L34" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M34" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B35" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C35" t="s">
         <v>15</v>
@@ -2189,57 +2192,57 @@
         <v>21</v>
       </c>
       <c r="J35" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K35" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="M35" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -2255,7 +2258,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(item-search): invalidate BUG-ISR-PCD-001 after owner-triggered LR-044 live re-verify — Category opens its dialog (walk no-op was a stale-ref instrument zero); TC-ISR-PCD-005 extended to Category (11 passed); claim swept across bug JSON, spec, TC-MD, 2 inventories, walk-evidence, master plan; CEO-M19 ledgered; workbooks rebuilt
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/encore/testcases/item-search/item-search-product-code.xlsx
+++ b/clients/encore/testcases/item-search/item-search-product-code.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="119">
   <si>
     <t>TC ID</t>
   </si>
@@ -223,7 +223,13 @@
     <t>The dialog opens with its first tab named "Class"</t>
   </si>
   <si>
-    <t>4. Close the dialog</t>
+    <t>4. Close the dialog, reopen the menu, click Category</t>
+  </si>
+  <si>
+    <t>The dialog opens with its first tab named "Category"</t>
+  </si>
+  <si>
+    <t>5. Close the dialog</t>
   </si>
   <si>
     <t>The grid is unchanged</t>
@@ -364,7 +370,7 @@
     <t>Last Updated: 2026-09-01</t>
   </si>
   <si>
-    <t>a5f7d6500d58722995e66601ec026824ea3e350a07badce9343a7a492d496f36</t>
+    <t>636a977849267dc2016113abf29c1c780ee08ec327c6f8ab32a1e036b3a6cf92</t>
   </si>
 </sst>
 </file>
@@ -753,7 +759,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M37"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1550,40 +1556,40 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20" t="s">
+        <v>25</v>
+      </c>
+      <c r="D20" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20" t="s">
+        <v>25</v>
+      </c>
+      <c r="G20" t="s">
+        <v>25</v>
+      </c>
+      <c r="H20" t="s">
+        <v>25</v>
+      </c>
+      <c r="I20" t="s">
+        <v>25</v>
+      </c>
+      <c r="J20" t="s">
+        <v>25</v>
+      </c>
+      <c r="K20" t="s">
         <v>71</v>
       </c>
-      <c r="B20" t="s">
+      <c r="L20" t="s">
         <v>72</v>
-      </c>
-      <c r="C20" t="s">
-        <v>15</v>
-      </c>
-      <c r="D20" t="s">
-        <v>16</v>
-      </c>
-      <c r="E20" t="s">
-        <v>17</v>
-      </c>
-      <c r="F20" t="s">
-        <v>18</v>
-      </c>
-      <c r="G20" t="s">
-        <v>19</v>
-      </c>
-      <c r="H20" t="s">
-        <v>20</v>
-      </c>
-      <c r="I20" t="s">
-        <v>21</v>
-      </c>
-      <c r="J20" t="s">
-        <v>30</v>
-      </c>
-      <c r="K20" t="s">
-        <v>73</v>
-      </c>
-      <c r="L20" t="s">
-        <v>74</v>
       </c>
       <c r="M20" t="s">
         <v>25</v>
@@ -1591,34 +1597,34 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>73</v>
       </c>
       <c r="B21" t="s">
-        <v>25</v>
+        <v>74</v>
       </c>
       <c r="C21" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D21" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E21" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F21" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="G21" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="H21" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I21" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J21" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="K21" t="s">
         <v>75</v>
@@ -1703,10 +1709,10 @@
         <v>25</v>
       </c>
       <c r="K23" t="s">
-        <v>37</v>
+        <v>79</v>
       </c>
       <c r="L23" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="M23" t="s">
         <v>25</v>
@@ -1714,40 +1720,40 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="B24" t="s">
+        <v>25</v>
+      </c>
+      <c r="C24" t="s">
+        <v>25</v>
+      </c>
+      <c r="D24" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" t="s">
+        <v>25</v>
+      </c>
+      <c r="F24" t="s">
+        <v>25</v>
+      </c>
+      <c r="G24" t="s">
+        <v>25</v>
+      </c>
+      <c r="H24" t="s">
+        <v>25</v>
+      </c>
+      <c r="I24" t="s">
+        <v>25</v>
+      </c>
+      <c r="J24" t="s">
+        <v>25</v>
+      </c>
+      <c r="K24" t="s">
+        <v>37</v>
+      </c>
+      <c r="L24" t="s">
         <v>81</v>
-      </c>
-      <c r="C24" t="s">
-        <v>15</v>
-      </c>
-      <c r="D24" t="s">
-        <v>16</v>
-      </c>
-      <c r="E24" t="s">
-        <v>17</v>
-      </c>
-      <c r="F24" t="s">
-        <v>18</v>
-      </c>
-      <c r="G24" t="s">
-        <v>19</v>
-      </c>
-      <c r="H24" t="s">
-        <v>20</v>
-      </c>
-      <c r="I24" t="s">
-        <v>21</v>
-      </c>
-      <c r="J24" t="s">
-        <v>82</v>
-      </c>
-      <c r="K24" t="s">
-        <v>83</v>
-      </c>
-      <c r="L24" t="s">
-        <v>84</v>
       </c>
       <c r="M24" t="s">
         <v>25</v>
@@ -1755,34 +1761,34 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>25</v>
+        <v>82</v>
       </c>
       <c r="B25" t="s">
-        <v>25</v>
+        <v>83</v>
       </c>
       <c r="C25" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D25" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E25" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F25" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="G25" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="H25" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I25" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J25" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="K25" t="s">
         <v>85</v>
@@ -1878,40 +1884,40 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B28" t="s">
+        <v>25</v>
+      </c>
+      <c r="C28" t="s">
+        <v>25</v>
+      </c>
+      <c r="D28" t="s">
+        <v>25</v>
+      </c>
+      <c r="E28" t="s">
+        <v>25</v>
+      </c>
+      <c r="F28" t="s">
+        <v>25</v>
+      </c>
+      <c r="G28" t="s">
+        <v>25</v>
+      </c>
+      <c r="H28" t="s">
+        <v>25</v>
+      </c>
+      <c r="I28" t="s">
+        <v>25</v>
+      </c>
+      <c r="J28" t="s">
+        <v>25</v>
+      </c>
+      <c r="K28" t="s">
         <v>91</v>
       </c>
-      <c r="B28" t="s">
+      <c r="L28" t="s">
         <v>92</v>
-      </c>
-      <c r="C28" t="s">
-        <v>15</v>
-      </c>
-      <c r="D28" t="s">
-        <v>16</v>
-      </c>
-      <c r="E28" t="s">
-        <v>17</v>
-      </c>
-      <c r="F28" t="s">
-        <v>18</v>
-      </c>
-      <c r="G28" t="s">
-        <v>19</v>
-      </c>
-      <c r="H28" t="s">
-        <v>20</v>
-      </c>
-      <c r="I28" t="s">
-        <v>21</v>
-      </c>
-      <c r="J28" t="s">
-        <v>62</v>
-      </c>
-      <c r="K28" t="s">
-        <v>93</v>
-      </c>
-      <c r="L28" t="s">
-        <v>64</v>
       </c>
       <c r="M28" t="s">
         <v>25</v>
@@ -1919,40 +1925,40 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>25</v>
+        <v>93</v>
       </c>
       <c r="B29" t="s">
-        <v>25</v>
+        <v>94</v>
       </c>
       <c r="C29" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D29" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E29" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F29" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="G29" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="H29" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I29" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J29" t="s">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="K29" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L29" t="s">
-        <v>95</v>
+        <v>64</v>
       </c>
       <c r="M29" t="s">
         <v>25</v>
@@ -1993,7 +1999,7 @@
         <v>96</v>
       </c>
       <c r="L30" t="s">
-        <v>70</v>
+        <v>97</v>
       </c>
       <c r="M30" t="s">
         <v>25</v>
@@ -2001,40 +2007,40 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>97</v>
+        <v>25</v>
       </c>
       <c r="B31" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" t="s">
+        <v>25</v>
+      </c>
+      <c r="D31" t="s">
+        <v>25</v>
+      </c>
+      <c r="E31" t="s">
+        <v>25</v>
+      </c>
+      <c r="F31" t="s">
+        <v>25</v>
+      </c>
+      <c r="G31" t="s">
+        <v>25</v>
+      </c>
+      <c r="H31" t="s">
+        <v>25</v>
+      </c>
+      <c r="I31" t="s">
+        <v>25</v>
+      </c>
+      <c r="J31" t="s">
+        <v>25</v>
+      </c>
+      <c r="K31" t="s">
         <v>98</v>
       </c>
-      <c r="C31" t="s">
-        <v>15</v>
-      </c>
-      <c r="D31" t="s">
-        <v>16</v>
-      </c>
-      <c r="E31" t="s">
-        <v>17</v>
-      </c>
-      <c r="F31" t="s">
-        <v>18</v>
-      </c>
-      <c r="G31" t="s">
-        <v>19</v>
-      </c>
-      <c r="H31" t="s">
-        <v>20</v>
-      </c>
-      <c r="I31" t="s">
-        <v>21</v>
-      </c>
-      <c r="J31" t="s">
-        <v>30</v>
-      </c>
-      <c r="K31" t="s">
-        <v>99</v>
-      </c>
       <c r="L31" t="s">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="M31" t="s">
         <v>25</v>
@@ -2042,34 +2048,34 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>25</v>
+        <v>99</v>
       </c>
       <c r="B32" t="s">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="C32" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D32" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E32" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F32" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="G32" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="H32" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I32" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J32" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="K32" t="s">
         <v>101</v>
@@ -2165,84 +2171,125 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>25</v>
+      </c>
+      <c r="B35" t="s">
+        <v>25</v>
+      </c>
+      <c r="C35" t="s">
+        <v>25</v>
+      </c>
+      <c r="D35" t="s">
+        <v>25</v>
+      </c>
+      <c r="E35" t="s">
+        <v>25</v>
+      </c>
+      <c r="F35" t="s">
+        <v>25</v>
+      </c>
+      <c r="G35" t="s">
+        <v>25</v>
+      </c>
+      <c r="H35" t="s">
+        <v>25</v>
+      </c>
+      <c r="I35" t="s">
+        <v>25</v>
+      </c>
+      <c r="J35" t="s">
+        <v>25</v>
+      </c>
+      <c r="K35" t="s">
         <v>107</v>
       </c>
-      <c r="B35" t="s">
+      <c r="L35" t="s">
         <v>108</v>
       </c>
-      <c r="C35" t="s">
+      <c r="M35" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>109</v>
+      </c>
+      <c r="B36" t="s">
+        <v>110</v>
+      </c>
+      <c r="C36" t="s">
         <v>15</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D36" t="s">
         <v>16</v>
       </c>
-      <c r="E35" t="s">
+      <c r="E36" t="s">
         <v>17</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F36" t="s">
         <v>18</v>
       </c>
-      <c r="G35" t="s">
+      <c r="G36" t="s">
         <v>19</v>
       </c>
-      <c r="H35" t="s">
+      <c r="H36" t="s">
         <v>20</v>
       </c>
-      <c r="I35" t="s">
+      <c r="I36" t="s">
         <v>21</v>
       </c>
-      <c r="J35" t="s">
+      <c r="J36" t="s">
         <v>30</v>
       </c>
-      <c r="K35" t="s">
-        <v>109</v>
-      </c>
-      <c r="L35" t="s">
-        <v>110</v>
-      </c>
-      <c r="M35" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A37" s="2" t="s">
+      <c r="K36" t="s">
         <v>111</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="L36" t="s">
         <v>112</v>
       </c>
-      <c r="C37" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="H37" s="2" t="s">
+      <c r="M36" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="I37" s="2" t="s">
+      <c r="B38" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="J37" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="K37" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L37" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M37" s="2" t="s">
+      <c r="C38" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H38" s="2" t="s">
         <v>115</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -2258,7 +2305,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>